<commit_message>
Add tab names to E04/E05 evidence references
E04 decisions: tab 2_Cisco Network Administrators rows 2538-2539; Netwrix log:
tabs 2-3 section REVOCATION EVIDENCE row 2976; AD extract: tabs 2-3 row 1639;
E05: tab 2.Cisco Network Administrators rows 3260, 3265. Applied to the testing
procedures, the design/sample-of-one document and E09; E00 MD5s refreshed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkbhuEGeprMY3UGeKiEnsh
</commit_message>
<xml_diff>
--- a/BSI.IT.27.C7/BSI.IT.27.C7_E00_Evidence Index.xlsx
+++ b/BSI.IT.27.C7/BSI.IT.27.C7_E00_Evidence Index.xlsx
@@ -617,7 +617,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>4a371954baaa764cf00e081cc51570aa</t>
+          <t>13ae14956684ea11ba1e60bf24c4e6f9</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>0c57096076ef641615e0acf82f87e79a</t>
+          <t>011708659aa4ec67fc480fa0f23c62b7</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>bc3b551c13bfc559b887c7f0d12f2d62</t>
+          <t>5e8d882d68f62eefa9209ee9ed19307f</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">

</xml_diff>